<commit_message>
comparing two months for summarised working hours
</commit_message>
<xml_diff>
--- a/grafiki/grafik_stany_2026_08.xlsx
+++ b/grafiki/grafik_stany_2026_08.xlsx
@@ -658,21 +658,21 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5,6,11,12,13,14,15,16,17,18,19,20,21,22,23,24,27,28,29,30</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -707,12 +707,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -727,12 +727,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -782,12 +782,12 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -821,16 +821,16 @@
         </is>
       </c>
       <c r="AK2" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="AL2" t="n">
-        <v>-160</v>
+        <v>-12</v>
       </c>
       <c r="AM2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AN2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AO2" t="n">
         <v>0</v>
@@ -863,21 +863,21 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -892,12 +892,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -937,12 +937,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -967,12 +967,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
@@ -1022,20 +1022,20 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="AL3" t="n">
-        <v>-160</v>
+        <v>-12</v>
       </c>
       <c r="AM3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AN3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO3" t="n">
         <v>0</v>
@@ -1068,11 +1068,11 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -1217,12 +1217,12 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1231,16 +1231,16 @@
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="AL4" t="n">
-        <v>-80</v>
+        <v>-12</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1273,11 +1273,11 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1292,12 +1292,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1312,12 +1312,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
@@ -1432,20 +1432,20 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="AL5" t="n">
-        <v>-160</v>
+        <v>-12</v>
       </c>
       <c r="AM5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AO5" t="n">
         <v>0</v>
@@ -1478,11 +1478,11 @@
         <v>0.5</v>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>12:D,13:D,18:N,19:N,20:N,25:N,26:N,27:N</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1572,12 +1572,12 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1641,16 +1641,16 @@
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="AL6" t="n">
-        <v>-80</v>
+        <v>-24</v>
       </c>
       <c r="AM6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1683,11 +1683,11 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5,6,16,23,28,29</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1702,12 +1702,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1797,12 +1797,12 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1827,12 +1827,12 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>D</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
@@ -1846,16 +1846,16 @@
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="AL7" t="n">
-        <v>-160</v>
+        <v>-24</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO7" t="n">
         <v>0</v>
@@ -1884,97 +1884,97 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AA8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AB8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AF8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AH8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AI8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>

</xml_diff>